<commit_message>
Import de la feuille hebdomadaire des dépenses (en-têtes « 3 شهر », rubriques, lignes sans libellé)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TqzfGGFyYFjt54rk5Bepb1
</commit_message>
<xml_diff>
--- a/canevas/caisse-donnees-reelles.xlsx
+++ b/canevas/caisse-donnees-reelles.xlsx
@@ -3580,7 +3580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H221"/>
+  <dimension ref="A1:H291"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3638,7 +3638,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>31/03/2025</t>
+          <t>01/03/2025</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -3648,7 +3648,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de mars 2025</t>
+          <t>أجرة الأسبوع من 03/03 إلى 09/03</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -3657,24 +3657,28 @@
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>1600</v>
+        <v>350</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 1</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par بوعزة</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>30/04/2025</t>
+          <t>08/03/2025</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -3684,7 +3688,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de avril 2025</t>
+          <t>أجرة الأسبوع من 10/03 إلى 16/03</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -3693,24 +3697,28 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1850</v>
+        <v>350</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 2</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>31/05/2025</t>
+          <t>15/03/2025</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -3720,7 +3728,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de mai 2025</t>
+          <t>أجرة الأسبوع من 17/03 إلى 23/03</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -3729,24 +3737,28 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>1450</v>
+        <v>350</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 3</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par بدر</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>30/06/2025</t>
+          <t>21/03/2025</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -3756,7 +3768,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de juin 2025</t>
+          <t>أجرة الأسبوع من 24/03 إلى 30/03</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -3765,24 +3777,28 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1600</v>
+        <v>350</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 4</t>
+        </is>
+      </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par الياس (عبد الرحمان)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>31/07/2025</t>
+          <t>31/03/2025</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3792,7 +3808,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de juillet 2025</t>
+          <t>أجرة الأسبوع من 31/03 إلى 06/04</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -3801,24 +3817,28 @@
         </is>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1750</v>
+        <v>350</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 5</t>
+        </is>
+      </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>31/08/2025</t>
+          <t>06/04/2025</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -3828,7 +3848,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de août 2025</t>
+          <t>أجرة الأسبوع من 07/04 إلى 13/04</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -3837,24 +3857,28 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 6</t>
+        </is>
+      </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>30/09/2025</t>
+          <t>11/04/2025</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3864,7 +3888,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de septembre 2025</t>
+          <t>أجرة الأسبوع من 14/04 إلى 20/04</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3873,24 +3897,28 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1750</v>
+        <v>350</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 7</t>
+        </is>
+      </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>31/10/2025</t>
+          <t>19/04/2025</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -3900,7 +3928,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de octobre 2025</t>
+          <t>أجرة الأسبوع من 21/04 إلى 27/04</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -3909,24 +3937,28 @@
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 8</t>
+        </is>
+      </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>30/11/2025</t>
+          <t>26/04/2025</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3936,7 +3968,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de novembre 2025</t>
+          <t>أجرة الأسبوع من 28/04 إلى 04/05</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -3945,24 +3977,28 @@
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 9</t>
+        </is>
+      </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par بدر</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>31/12/2025</t>
+          <t>04/05/2025</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -3972,7 +4008,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de décembre 2025</t>
+          <t>أجرة الأسبوع من 05/05 إلى 11/05</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -3981,24 +4017,28 @@
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1750</v>
+        <v>350</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 10</t>
+        </is>
+      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par الياس</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>31/01/2026</t>
+          <t>10/05/2025</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -4008,7 +4048,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de janvier 2026</t>
+          <t>أجرة الأسبوع من 12/05 إلى 18/05</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -4017,24 +4057,28 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>1750</v>
+        <v>350</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 11</t>
+        </is>
+      </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>28/02/2026</t>
+          <t>17/05/2025</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
@@ -4044,7 +4088,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de février 2026</t>
+          <t>أجرة الأسبوع من 19/05 إلى 25/05</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -4053,24 +4097,28 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 12</t>
+        </is>
+      </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par الياس</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>31/03/2026</t>
+          <t>23/05/2025</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -4080,7 +4128,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de mars 2026</t>
+          <t>أجرة الأسبوع من 26/05 إلى 01/06</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -4089,24 +4137,28 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 13</t>
+        </is>
+      </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>01/06/2025</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -4116,7 +4168,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de avril 2026</t>
+          <t>أجرة الأسبوع من 02/06 إلى 08/06</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -4125,24 +4177,28 @@
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 14</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>09/06/2025</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -4152,7 +4208,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de mai 2026</t>
+          <t>أجرة الأسبوع من 09/06 إلى 15/06</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -4161,24 +4217,28 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>1750</v>
+        <v>350</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 15</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>30/06/2026</t>
+          <t>14/06/2025</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -4188,7 +4248,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de juin 2026</t>
+          <t>أجرة الأسبوع من 16/06 إلى 22/06</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -4197,24 +4257,28 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 16</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -4224,7 +4288,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de juillet 2026</t>
+          <t>أجرة الأسبوع من 23/06 إلى 29/06</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -4233,24 +4297,28 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 17</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>31/08/2026</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
@@ -4260,7 +4328,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de août 2026</t>
+          <t>أجرة الأسبوع من 30/06 إلى 06/07</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -4269,24 +4337,28 @@
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>1750</v>
+        <v>350</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 18</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>30/09/2026</t>
+          <t>06/07/2025</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -4296,7 +4368,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de septembre 2026</t>
+          <t>أجرة الأسبوع من 07/07 إلى 13/07</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -4305,24 +4377,28 @@
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>1400</v>
+        <v>350</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 19</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>13/07/2025</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
@@ -4332,7 +4408,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Dépenses du mois de octobre 2026</t>
+          <t>أجرة الأسبوع من 14/07 إلى 20/07</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -4348,712 +4424,2660 @@
           <t>Espèces</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 20</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Total mensuel repris du fichier Excel</t>
+          <t>Payé par امحمد</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>20/07/2025</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 21/07 إلى 27/07</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 21</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
-      <c r="B23" s="2" t="n"/>
-      <c r="C23" s="2" t="n"/>
-      <c r="D23" s="2" t="n"/>
-      <c r="E23" s="3" t="n"/>
-      <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>26/07/2025</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 28/07 إلى 03/08</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 22</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="3" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n"/>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>02/08/2025</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 04/08 إلى 10/08</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 23</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="2" t="n"/>
-      <c r="G25" s="2" t="n"/>
-      <c r="H25" s="2" t="n"/>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>09/08/2025</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 11/08 إلى 17/08</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>400</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 24</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>17/08/2025</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 18/08 إلى 24/08</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 25</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Payé par عبد الرحمان</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="n"/>
-      <c r="H27" s="2" t="n"/>
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>26/08/2025</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 25/08 إلى 31/08</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 26</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
-      <c r="B28" s="2" t="n"/>
-      <c r="C28" s="2" t="n"/>
-      <c r="D28" s="2" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="n"/>
-      <c r="H28" s="2" t="n"/>
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>30/08/2025</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 01/09 إلى 07/09</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 27</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
-      <c r="B29" s="2" t="n"/>
-      <c r="C29" s="2" t="n"/>
-      <c r="D29" s="2" t="n"/>
-      <c r="E29" s="3" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="n"/>
-      <c r="H29" s="2" t="n"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>06/09/2025</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 08/09 إلى 14/09</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 28</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد · date corrigée (fichier : 06/08/2025)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
-      <c r="B30" s="2" t="n"/>
-      <c r="C30" s="2" t="n"/>
-      <c r="D30" s="2" t="n"/>
-      <c r="E30" s="3" t="n"/>
-      <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="n"/>
-      <c r="H30" s="2" t="n"/>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>13/09/2025</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 15/09 إلى 21/09</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 29</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="3" t="n"/>
-      <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-      <c r="H31" s="2" t="n"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>20/09/2025</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 22/09 إلى 28/09</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 30</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="3" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
-      <c r="H32" s="2" t="n"/>
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>27/09/2025</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 29/09 إلى 05/10</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 31</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
-      <c r="B33" s="2" t="n"/>
-      <c r="C33" s="2" t="n"/>
-      <c r="D33" s="2" t="n"/>
-      <c r="E33" s="3" t="n"/>
-      <c r="F33" s="2" t="n"/>
-      <c r="G33" s="2" t="n"/>
-      <c r="H33" s="2" t="n"/>
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>04/10/2025</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 06/10 إلى 12/10</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 32</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
-      <c r="B34" s="2" t="n"/>
-      <c r="C34" s="2" t="n"/>
-      <c r="D34" s="2" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="2" t="n"/>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>12/10/2025</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 13/10 إلى 19/10</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 33</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
-      <c r="B35" s="2" t="n"/>
-      <c r="C35" s="2" t="n"/>
-      <c r="D35" s="2" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="2" t="n"/>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>19/10/2025</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 20/10 إلى 26/10</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 34</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
-      <c r="B36" s="2" t="n"/>
-      <c r="C36" s="2" t="n"/>
-      <c r="D36" s="2" t="n"/>
-      <c r="E36" s="3" t="n"/>
-      <c r="F36" s="2" t="n"/>
-      <c r="G36" s="2" t="n"/>
-      <c r="H36" s="2" t="n"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>25/10/2025</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 27/10 إلى 02/11</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 35</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
-      <c r="B37" s="2" t="n"/>
-      <c r="C37" s="2" t="n"/>
-      <c r="D37" s="2" t="n"/>
-      <c r="E37" s="3" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="n"/>
-      <c r="H37" s="2" t="n"/>
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>01/11/2025</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 03/11 إلى 09/11</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 36</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
-      <c r="B38" s="2" t="n"/>
-      <c r="C38" s="2" t="n"/>
-      <c r="D38" s="2" t="n"/>
-      <c r="E38" s="3" t="n"/>
-      <c r="F38" s="2" t="n"/>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n"/>
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>09/11/2025</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 10/11 إلى 16/11</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 37</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
-      <c r="B39" s="2" t="n"/>
-      <c r="C39" s="2" t="n"/>
-      <c r="D39" s="2" t="n"/>
-      <c r="E39" s="3" t="n"/>
-      <c r="F39" s="2" t="n"/>
-      <c r="G39" s="2" t="n"/>
-      <c r="H39" s="2" t="n"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>15/11/2025</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 17/11 إلى 23/11</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 38</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
-      <c r="B40" s="2" t="n"/>
-      <c r="C40" s="2" t="n"/>
-      <c r="D40" s="2" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="2" t="n"/>
-      <c r="G40" s="2" t="n"/>
-      <c r="H40" s="2" t="n"/>
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>23/11/2025</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 24/11 إلى 30/11</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 39</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n"/>
-      <c r="B41" s="2" t="n"/>
-      <c r="C41" s="2" t="n"/>
-      <c r="D41" s="2" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="2" t="n"/>
-      <c r="G41" s="2" t="n"/>
-      <c r="H41" s="2" t="n"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>29/11/2025</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 01/12 إلى 07/12</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 40</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
-      <c r="B42" s="2" t="n"/>
-      <c r="C42" s="2" t="n"/>
-      <c r="D42" s="2" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="2" t="n"/>
-      <c r="G42" s="2" t="n"/>
-      <c r="H42" s="2" t="n"/>
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>06/12/2025</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 08/12 إلى 14/12</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 41</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>Payé par مهدي</t>
+        </is>
+      </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
-      <c r="B43" s="2" t="n"/>
-      <c r="C43" s="2" t="n"/>
-      <c r="D43" s="2" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="n"/>
-      <c r="H43" s="2" t="n"/>
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>14/12/2025</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 15/12 إلى 21/12</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 42</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
-      <c r="C44" s="2" t="n"/>
-      <c r="D44" s="2" t="n"/>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="n"/>
-      <c r="H44" s="2" t="n"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>22/12/2025</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 22/12 إلى 28/12</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 43</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
-      <c r="B45" s="2" t="n"/>
-      <c r="C45" s="2" t="n"/>
-      <c r="D45" s="2" t="n"/>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="2" t="n"/>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>28/12/2025</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الأسبوع من 29/12 إلى 04/01 (2026)</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 44</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
-      <c r="B46" s="2" t="n"/>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="n"/>
-      <c r="E46" s="3" t="n"/>
-      <c r="F46" s="2" t="n"/>
-      <c r="G46" s="2" t="n"/>
-      <c r="H46" s="2" t="n"/>
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>03/01/2026</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 1</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
-      <c r="B47" s="2" t="n"/>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="n"/>
-      <c r="E47" s="3" t="n"/>
-      <c r="F47" s="2" t="n"/>
-      <c r="G47" s="2" t="n"/>
-      <c r="H47" s="2" t="n"/>
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>11/01/2026</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 2</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
-      <c r="C48" s="2" t="n"/>
-      <c r="D48" s="2" t="n"/>
-      <c r="E48" s="3" t="n"/>
-      <c r="F48" s="2" t="n"/>
-      <c r="G48" s="2" t="n"/>
-      <c r="H48" s="2" t="n"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>18/01/2026</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 3</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n"/>
-      <c r="B49" s="2" t="n"/>
-      <c r="C49" s="2" t="n"/>
-      <c r="D49" s="2" t="n"/>
-      <c r="E49" s="3" t="n"/>
-      <c r="F49" s="2" t="n"/>
-      <c r="G49" s="2" t="n"/>
-      <c r="H49" s="2" t="n"/>
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>24/01/2026</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 4</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n"/>
-      <c r="B50" s="2" t="n"/>
-      <c r="C50" s="2" t="n"/>
-      <c r="D50" s="2" t="n"/>
-      <c r="E50" s="3" t="n"/>
-      <c r="F50" s="2" t="n"/>
-      <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="n"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>31/01/2026</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 5</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بوعزة</t>
+        </is>
+      </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n"/>
-      <c r="B51" s="2" t="n"/>
-      <c r="C51" s="2" t="n"/>
-      <c r="D51" s="2" t="n"/>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="2" t="n"/>
-      <c r="G51" s="2" t="n"/>
-      <c r="H51" s="2" t="n"/>
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>07/02/2026</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 6</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
-      <c r="B52" s="2" t="n"/>
-      <c r="C52" s="2" t="n"/>
-      <c r="D52" s="2" t="n"/>
-      <c r="E52" s="3" t="n"/>
-      <c r="F52" s="2" t="n"/>
-      <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="n"/>
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>15/02/2026</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 7</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بوعزة</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
-      <c r="B53" s="2" t="n"/>
-      <c r="C53" s="2" t="n"/>
-      <c r="D53" s="2" t="n"/>
-      <c r="E53" s="3" t="n"/>
-      <c r="F53" s="2" t="n"/>
-      <c r="G53" s="2" t="n"/>
-      <c r="H53" s="2" t="n"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>21/02/2026</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 8</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
-      <c r="B54" s="2" t="n"/>
-      <c r="C54" s="2" t="n"/>
-      <c r="D54" s="2" t="n"/>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="2" t="n"/>
-      <c r="H54" s="2" t="n"/>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>28/02/2026</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 9</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="n"/>
-      <c r="D55" s="2" t="n"/>
-      <c r="E55" s="3" t="n"/>
-      <c r="F55" s="2" t="n"/>
-      <c r="G55" s="2" t="n"/>
-      <c r="H55" s="2" t="n"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>07/03/2026</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 10</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n"/>
-      <c r="B56" s="2" t="n"/>
-      <c r="C56" s="2" t="n"/>
-      <c r="D56" s="2" t="n"/>
-      <c r="E56" s="3" t="n"/>
-      <c r="F56" s="2" t="n"/>
-      <c r="G56" s="2" t="n"/>
-      <c r="H56" s="2" t="n"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 11</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بوعزة</t>
+        </is>
+      </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n"/>
-      <c r="B57" s="2" t="n"/>
-      <c r="C57" s="2" t="n"/>
-      <c r="D57" s="2" t="n"/>
-      <c r="E57" s="3" t="n"/>
-      <c r="F57" s="2" t="n"/>
-      <c r="G57" s="2" t="n"/>
-      <c r="H57" s="2" t="n"/>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 12</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بوعزة</t>
+        </is>
+      </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
-      <c r="C58" s="2" t="n"/>
-      <c r="D58" s="2" t="n"/>
-      <c r="E58" s="3" t="n"/>
-      <c r="F58" s="2" t="n"/>
-      <c r="G58" s="2" t="n"/>
-      <c r="H58" s="2" t="n"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>28/03/2026</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Semaine 13</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
-      <c r="B59" s="2" t="n"/>
-      <c r="C59" s="2" t="n"/>
-      <c r="D59" s="2" t="n"/>
-      <c r="E59" s="3" t="n"/>
-      <c r="F59" s="2" t="n"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G59" s="2" t="n"/>
-      <c r="H59" s="2" t="n"/>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
-      <c r="B60" s="2" t="n"/>
-      <c r="C60" s="2" t="n"/>
-      <c r="D60" s="2" t="n"/>
-      <c r="E60" s="3" t="n"/>
-      <c r="F60" s="2" t="n"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G60" s="2" t="n"/>
-      <c r="H60" s="2" t="n"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="2" t="n"/>
-      <c r="C61" s="2" t="n"/>
-      <c r="D61" s="2" t="n"/>
-      <c r="E61" s="3" t="n"/>
-      <c r="F61" s="2" t="n"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G61" s="2" t="n"/>
-      <c r="H61" s="2" t="n"/>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n"/>
-      <c r="B62" s="2" t="n"/>
-      <c r="C62" s="2" t="n"/>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="3" t="n"/>
-      <c r="F62" s="2" t="n"/>
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>25/04/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G62" s="2" t="n"/>
-      <c r="H62" s="2" t="n"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
-      <c r="B63" s="2" t="n"/>
-      <c r="C63" s="2" t="n"/>
-      <c r="D63" s="2" t="n"/>
-      <c r="E63" s="3" t="n"/>
-      <c r="F63" s="2" t="n"/>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>02/05/2026</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G63" s="2" t="n"/>
-      <c r="H63" s="2" t="n"/>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
-      <c r="C64" s="2" t="n"/>
-      <c r="D64" s="2" t="n"/>
-      <c r="E64" s="3" t="n"/>
-      <c r="F64" s="2" t="n"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>10/05/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G64" s="2" t="n"/>
-      <c r="H64" s="2" t="n"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس</t>
+        </is>
+      </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n"/>
-      <c r="B65" s="2" t="n"/>
-      <c r="C65" s="2" t="n"/>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="3" t="n"/>
-      <c r="F65" s="2" t="n"/>
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>16/05/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="n"/>
-      <c r="H65" s="2" t="n"/>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n"/>
-      <c r="B66" s="2" t="n"/>
-      <c r="C66" s="2" t="n"/>
-      <c r="D66" s="2" t="n"/>
-      <c r="E66" s="3" t="n"/>
-      <c r="F66" s="2" t="n"/>
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>23/05/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="n"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n"/>
-      <c r="B67" s="2" t="n"/>
-      <c r="C67" s="2" t="n"/>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="3" t="n"/>
-      <c r="F67" s="2" t="n"/>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>30/05/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G67" s="2" t="n"/>
-      <c r="H67" s="2" t="n"/>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n"/>
-      <c r="B68" s="2" t="n"/>
-      <c r="C68" s="2" t="n"/>
-      <c r="D68" s="2" t="n"/>
-      <c r="E68" s="3" t="n"/>
-      <c r="F68" s="2" t="n"/>
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G68" s="2" t="n"/>
-      <c r="H68" s="2" t="n"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بدر</t>
+        </is>
+      </c>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
-      <c r="B69" s="2" t="n"/>
-      <c r="C69" s="2" t="n"/>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="3" t="n"/>
-      <c r="F69" s="2" t="n"/>
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>13/06/2026</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G69" s="2" t="n"/>
-      <c r="H69" s="2" t="n"/>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بدر</t>
+        </is>
+      </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n"/>
-      <c r="B70" s="2" t="n"/>
-      <c r="C70" s="2" t="n"/>
-      <c r="D70" s="2" t="n"/>
-      <c r="E70" s="3" t="n"/>
-      <c r="F70" s="2" t="n"/>
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>20/06/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G70" s="2" t="n"/>
-      <c r="H70" s="2" t="n"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n"/>
-      <c r="B71" s="2" t="n"/>
-      <c r="C71" s="2" t="n"/>
-      <c r="D71" s="2" t="n"/>
-      <c r="E71" s="3" t="n"/>
-      <c r="F71" s="2" t="n"/>
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>27/06/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G71" s="2" t="n"/>
-      <c r="H71" s="2" t="n"/>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n"/>
-      <c r="B72" s="2" t="n"/>
-      <c r="C72" s="2" t="n"/>
-      <c r="D72" s="2" t="n"/>
-      <c r="E72" s="3" t="n"/>
-      <c r="F72" s="2" t="n"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>04/07/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="n"/>
-      <c r="H72" s="2" t="n"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n"/>
-      <c r="B73" s="2" t="n"/>
-      <c r="C73" s="2" t="n"/>
-      <c r="D73" s="2" t="n"/>
-      <c r="E73" s="3" t="n"/>
-      <c r="F73" s="2" t="n"/>
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="n"/>
-      <c r="H73" s="2" t="n"/>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n"/>
-      <c r="B74" s="2" t="n"/>
-      <c r="C74" s="2" t="n"/>
-      <c r="D74" s="2" t="n"/>
-      <c r="E74" s="3" t="n"/>
-      <c r="F74" s="2" t="n"/>
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>18/07/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G74" s="2" t="n"/>
-      <c r="H74" s="2" t="n"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n"/>
-      <c r="B75" s="2" t="n"/>
-      <c r="C75" s="2" t="n"/>
-      <c r="D75" s="2" t="n"/>
-      <c r="E75" s="3" t="n"/>
-      <c r="F75" s="2" t="n"/>
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>26/07/2026</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="n"/>
-      <c r="H75" s="2" t="n"/>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n"/>
-      <c r="B76" s="2" t="n"/>
-      <c r="C76" s="2" t="n"/>
-      <c r="D76" s="2" t="n"/>
-      <c r="E76" s="3" t="n"/>
-      <c r="F76" s="2" t="n"/>
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>01/08/2026</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G76" s="2" t="n"/>
-      <c r="H76" s="2" t="n"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>Payé par الياس ز</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n"/>
-      <c r="B77" s="2" t="n"/>
-      <c r="C77" s="2" t="n"/>
-      <c r="D77" s="2" t="n"/>
-      <c r="E77" s="3" t="n"/>
-      <c r="F77" s="2" t="n"/>
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>08/08/2026</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="n"/>
-      <c r="H77" s="2" t="n"/>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بدر</t>
+        </is>
+      </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n"/>
-      <c r="B78" s="2" t="n"/>
-      <c r="C78" s="2" t="n"/>
-      <c r="D78" s="2" t="n"/>
-      <c r="E78" s="3" t="n"/>
-      <c r="F78" s="2" t="n"/>
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>16/08/2026</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G78" s="2" t="n"/>
-      <c r="H78" s="2" t="n"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n"/>
-      <c r="B79" s="2" t="n"/>
-      <c r="C79" s="2" t="n"/>
-      <c r="D79" s="2" t="n"/>
-      <c r="E79" s="3" t="n"/>
-      <c r="F79" s="2" t="n"/>
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E79" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G79" s="2" t="n"/>
-      <c r="H79" s="2" t="n"/>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n"/>
-      <c r="B80" s="2" t="n"/>
-      <c r="C80" s="2" t="n"/>
-      <c r="D80" s="2" t="n"/>
-      <c r="E80" s="3" t="n"/>
-      <c r="F80" s="2" t="n"/>
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G80" s="2" t="n"/>
-      <c r="H80" s="2" t="n"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n"/>
-      <c r="B81" s="2" t="n"/>
-      <c r="C81" s="2" t="n"/>
-      <c r="D81" s="2" t="n"/>
-      <c r="E81" s="3" t="n"/>
-      <c r="F81" s="2" t="n"/>
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>05/09/2026</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E81" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G81" s="2" t="n"/>
-      <c r="H81" s="2" t="n"/>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n"/>
-      <c r="B82" s="2" t="n"/>
-      <c r="C82" s="2" t="n"/>
-      <c r="D82" s="2" t="n"/>
-      <c r="E82" s="3" t="n"/>
-      <c r="F82" s="2" t="n"/>
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>13/09/2026</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G82" s="2" t="n"/>
-      <c r="H82" s="2" t="n"/>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n"/>
-      <c r="B83" s="2" t="n"/>
-      <c r="C83" s="2" t="n"/>
-      <c r="D83" s="2" t="n"/>
-      <c r="E83" s="3" t="n"/>
-      <c r="F83" s="2" t="n"/>
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>19/09/2026</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E83" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G83" s="2" t="n"/>
-      <c r="H83" s="2" t="n"/>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n"/>
-      <c r="B84" s="2" t="n"/>
-      <c r="C84" s="2" t="n"/>
-      <c r="D84" s="2" t="n"/>
-      <c r="E84" s="3" t="n"/>
-      <c r="F84" s="2" t="n"/>
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>26/09/2026</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G84" s="2" t="n"/>
-      <c r="H84" s="2" t="n"/>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n"/>
-      <c r="B85" s="2" t="n"/>
-      <c r="C85" s="2" t="n"/>
-      <c r="D85" s="2" t="n"/>
-      <c r="E85" s="3" t="n"/>
-      <c r="F85" s="2" t="n"/>
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>03/10/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>Paiement du personnel</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>أجرة الحارس الأسبوعية</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Gardien</t>
+        </is>
+      </c>
+      <c r="E85" s="3" t="n">
+        <v>350</v>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G85" s="2" t="n"/>
-      <c r="H85" s="2" t="n"/>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n"/>
-      <c r="B86" s="2" t="n"/>
-      <c r="C86" s="2" t="n"/>
-      <c r="D86" s="2" t="n"/>
-      <c r="E86" s="3" t="n"/>
-      <c r="F86" s="2" t="n"/>
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>08/03/2025</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>Charges communes</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>تعبئة عداد الكهرباء</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G86" s="2" t="n"/>
-      <c r="H86" s="2" t="n"/>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n"/>
-      <c r="B87" s="2" t="n"/>
-      <c r="C87" s="2" t="n"/>
-      <c r="D87" s="2" t="n"/>
-      <c r="E87" s="3" t="n"/>
-      <c r="F87" s="2" t="n"/>
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>30/03/2025</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>Charges communes</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>تعبئة عداد الكهرباء</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G87" s="2" t="n"/>
-      <c r="H87" s="2" t="n"/>
+      <c r="H87" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n"/>
-      <c r="B88" s="2" t="n"/>
-      <c r="C88" s="2" t="n"/>
-      <c r="D88" s="2" t="n"/>
-      <c r="E88" s="3" t="n"/>
-      <c r="F88" s="2" t="n"/>
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>26/04/2025</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>Charges communes</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>تعبئة عداد الكهرباء</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G88" s="2" t="n"/>
-      <c r="H88" s="2" t="n"/>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Payé par بدر</t>
+        </is>
+      </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n"/>
-      <c r="B89" s="2" t="n"/>
-      <c r="C89" s="2" t="n"/>
-      <c r="D89" s="2" t="n"/>
-      <c r="E89" s="3" t="n"/>
-      <c r="F89" s="2" t="n"/>
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>22/05/2025</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>Charges communes</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>تعبئة عداد الكهرباء</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr"/>
+      <c r="E89" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G89" s="2" t="n"/>
-      <c r="H89" s="2" t="n"/>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n"/>
-      <c r="B90" s="2" t="n"/>
-      <c r="C90" s="2" t="n"/>
-      <c r="D90" s="2" t="n"/>
-      <c r="E90" s="3" t="n"/>
-      <c r="F90" s="2" t="n"/>
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>06/06/2025</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Charges communes</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>تعبئة عداد الكهرباء</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr"/>
+      <c r="E90" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G90" s="2" t="n"/>
-      <c r="H90" s="2" t="n"/>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n"/>
-      <c r="B91" s="2" t="n"/>
-      <c r="C91" s="2" t="n"/>
-      <c r="D91" s="2" t="n"/>
-      <c r="E91" s="3" t="n"/>
-      <c r="F91" s="2" t="n"/>
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>25/06/2025</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>Charges communes</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>تعبئة عداد الكهرباء</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>Espèces</t>
+        </is>
+      </c>
       <c r="G91" s="2" t="n"/>
-      <c r="H91" s="2" t="n"/>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>Payé par امحمد</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n"/>
@@ -6354,6 +8378,706 @@
       <c r="F221" s="2" t="n"/>
       <c r="G221" s="2" t="n"/>
       <c r="H221" s="2" t="n"/>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="n"/>
+      <c r="B222" s="2" t="n"/>
+      <c r="C222" s="2" t="n"/>
+      <c r="D222" s="2" t="n"/>
+      <c r="E222" s="3" t="n"/>
+      <c r="F222" s="2" t="n"/>
+      <c r="G222" s="2" t="n"/>
+      <c r="H222" s="2" t="n"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="n"/>
+      <c r="B223" s="2" t="n"/>
+      <c r="C223" s="2" t="n"/>
+      <c r="D223" s="2" t="n"/>
+      <c r="E223" s="3" t="n"/>
+      <c r="F223" s="2" t="n"/>
+      <c r="G223" s="2" t="n"/>
+      <c r="H223" s="2" t="n"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="n"/>
+      <c r="B224" s="2" t="n"/>
+      <c r="C224" s="2" t="n"/>
+      <c r="D224" s="2" t="n"/>
+      <c r="E224" s="3" t="n"/>
+      <c r="F224" s="2" t="n"/>
+      <c r="G224" s="2" t="n"/>
+      <c r="H224" s="2" t="n"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="n"/>
+      <c r="B225" s="2" t="n"/>
+      <c r="C225" s="2" t="n"/>
+      <c r="D225" s="2" t="n"/>
+      <c r="E225" s="3" t="n"/>
+      <c r="F225" s="2" t="n"/>
+      <c r="G225" s="2" t="n"/>
+      <c r="H225" s="2" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="n"/>
+      <c r="B226" s="2" t="n"/>
+      <c r="C226" s="2" t="n"/>
+      <c r="D226" s="2" t="n"/>
+      <c r="E226" s="3" t="n"/>
+      <c r="F226" s="2" t="n"/>
+      <c r="G226" s="2" t="n"/>
+      <c r="H226" s="2" t="n"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="n"/>
+      <c r="B227" s="2" t="n"/>
+      <c r="C227" s="2" t="n"/>
+      <c r="D227" s="2" t="n"/>
+      <c r="E227" s="3" t="n"/>
+      <c r="F227" s="2" t="n"/>
+      <c r="G227" s="2" t="n"/>
+      <c r="H227" s="2" t="n"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="n"/>
+      <c r="B228" s="2" t="n"/>
+      <c r="C228" s="2" t="n"/>
+      <c r="D228" s="2" t="n"/>
+      <c r="E228" s="3" t="n"/>
+      <c r="F228" s="2" t="n"/>
+      <c r="G228" s="2" t="n"/>
+      <c r="H228" s="2" t="n"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="n"/>
+      <c r="B229" s="2" t="n"/>
+      <c r="C229" s="2" t="n"/>
+      <c r="D229" s="2" t="n"/>
+      <c r="E229" s="3" t="n"/>
+      <c r="F229" s="2" t="n"/>
+      <c r="G229" s="2" t="n"/>
+      <c r="H229" s="2" t="n"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="n"/>
+      <c r="B230" s="2" t="n"/>
+      <c r="C230" s="2" t="n"/>
+      <c r="D230" s="2" t="n"/>
+      <c r="E230" s="3" t="n"/>
+      <c r="F230" s="2" t="n"/>
+      <c r="G230" s="2" t="n"/>
+      <c r="H230" s="2" t="n"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="n"/>
+      <c r="B231" s="2" t="n"/>
+      <c r="C231" s="2" t="n"/>
+      <c r="D231" s="2" t="n"/>
+      <c r="E231" s="3" t="n"/>
+      <c r="F231" s="2" t="n"/>
+      <c r="G231" s="2" t="n"/>
+      <c r="H231" s="2" t="n"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="n"/>
+      <c r="B232" s="2" t="n"/>
+      <c r="C232" s="2" t="n"/>
+      <c r="D232" s="2" t="n"/>
+      <c r="E232" s="3" t="n"/>
+      <c r="F232" s="2" t="n"/>
+      <c r="G232" s="2" t="n"/>
+      <c r="H232" s="2" t="n"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="n"/>
+      <c r="B233" s="2" t="n"/>
+      <c r="C233" s="2" t="n"/>
+      <c r="D233" s="2" t="n"/>
+      <c r="E233" s="3" t="n"/>
+      <c r="F233" s="2" t="n"/>
+      <c r="G233" s="2" t="n"/>
+      <c r="H233" s="2" t="n"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="n"/>
+      <c r="B234" s="2" t="n"/>
+      <c r="C234" s="2" t="n"/>
+      <c r="D234" s="2" t="n"/>
+      <c r="E234" s="3" t="n"/>
+      <c r="F234" s="2" t="n"/>
+      <c r="G234" s="2" t="n"/>
+      <c r="H234" s="2" t="n"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="n"/>
+      <c r="B235" s="2" t="n"/>
+      <c r="C235" s="2" t="n"/>
+      <c r="D235" s="2" t="n"/>
+      <c r="E235" s="3" t="n"/>
+      <c r="F235" s="2" t="n"/>
+      <c r="G235" s="2" t="n"/>
+      <c r="H235" s="2" t="n"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="n"/>
+      <c r="B236" s="2" t="n"/>
+      <c r="C236" s="2" t="n"/>
+      <c r="D236" s="2" t="n"/>
+      <c r="E236" s="3" t="n"/>
+      <c r="F236" s="2" t="n"/>
+      <c r="G236" s="2" t="n"/>
+      <c r="H236" s="2" t="n"/>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="n"/>
+      <c r="B237" s="2" t="n"/>
+      <c r="C237" s="2" t="n"/>
+      <c r="D237" s="2" t="n"/>
+      <c r="E237" s="3" t="n"/>
+      <c r="F237" s="2" t="n"/>
+      <c r="G237" s="2" t="n"/>
+      <c r="H237" s="2" t="n"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="n"/>
+      <c r="B238" s="2" t="n"/>
+      <c r="C238" s="2" t="n"/>
+      <c r="D238" s="2" t="n"/>
+      <c r="E238" s="3" t="n"/>
+      <c r="F238" s="2" t="n"/>
+      <c r="G238" s="2" t="n"/>
+      <c r="H238" s="2" t="n"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="n"/>
+      <c r="B239" s="2" t="n"/>
+      <c r="C239" s="2" t="n"/>
+      <c r="D239" s="2" t="n"/>
+      <c r="E239" s="3" t="n"/>
+      <c r="F239" s="2" t="n"/>
+      <c r="G239" s="2" t="n"/>
+      <c r="H239" s="2" t="n"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="n"/>
+      <c r="B240" s="2" t="n"/>
+      <c r="C240" s="2" t="n"/>
+      <c r="D240" s="2" t="n"/>
+      <c r="E240" s="3" t="n"/>
+      <c r="F240" s="2" t="n"/>
+      <c r="G240" s="2" t="n"/>
+      <c r="H240" s="2" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="n"/>
+      <c r="B241" s="2" t="n"/>
+      <c r="C241" s="2" t="n"/>
+      <c r="D241" s="2" t="n"/>
+      <c r="E241" s="3" t="n"/>
+      <c r="F241" s="2" t="n"/>
+      <c r="G241" s="2" t="n"/>
+      <c r="H241" s="2" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="n"/>
+      <c r="B242" s="2" t="n"/>
+      <c r="C242" s="2" t="n"/>
+      <c r="D242" s="2" t="n"/>
+      <c r="E242" s="3" t="n"/>
+      <c r="F242" s="2" t="n"/>
+      <c r="G242" s="2" t="n"/>
+      <c r="H242" s="2" t="n"/>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="n"/>
+      <c r="B243" s="2" t="n"/>
+      <c r="C243" s="2" t="n"/>
+      <c r="D243" s="2" t="n"/>
+      <c r="E243" s="3" t="n"/>
+      <c r="F243" s="2" t="n"/>
+      <c r="G243" s="2" t="n"/>
+      <c r="H243" s="2" t="n"/>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="n"/>
+      <c r="B244" s="2" t="n"/>
+      <c r="C244" s="2" t="n"/>
+      <c r="D244" s="2" t="n"/>
+      <c r="E244" s="3" t="n"/>
+      <c r="F244" s="2" t="n"/>
+      <c r="G244" s="2" t="n"/>
+      <c r="H244" s="2" t="n"/>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="n"/>
+      <c r="B245" s="2" t="n"/>
+      <c r="C245" s="2" t="n"/>
+      <c r="D245" s="2" t="n"/>
+      <c r="E245" s="3" t="n"/>
+      <c r="F245" s="2" t="n"/>
+      <c r="G245" s="2" t="n"/>
+      <c r="H245" s="2" t="n"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="n"/>
+      <c r="B246" s="2" t="n"/>
+      <c r="C246" s="2" t="n"/>
+      <c r="D246" s="2" t="n"/>
+      <c r="E246" s="3" t="n"/>
+      <c r="F246" s="2" t="n"/>
+      <c r="G246" s="2" t="n"/>
+      <c r="H246" s="2" t="n"/>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="n"/>
+      <c r="B247" s="2" t="n"/>
+      <c r="C247" s="2" t="n"/>
+      <c r="D247" s="2" t="n"/>
+      <c r="E247" s="3" t="n"/>
+      <c r="F247" s="2" t="n"/>
+      <c r="G247" s="2" t="n"/>
+      <c r="H247" s="2" t="n"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="n"/>
+      <c r="B248" s="2" t="n"/>
+      <c r="C248" s="2" t="n"/>
+      <c r="D248" s="2" t="n"/>
+      <c r="E248" s="3" t="n"/>
+      <c r="F248" s="2" t="n"/>
+      <c r="G248" s="2" t="n"/>
+      <c r="H248" s="2" t="n"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="n"/>
+      <c r="B249" s="2" t="n"/>
+      <c r="C249" s="2" t="n"/>
+      <c r="D249" s="2" t="n"/>
+      <c r="E249" s="3" t="n"/>
+      <c r="F249" s="2" t="n"/>
+      <c r="G249" s="2" t="n"/>
+      <c r="H249" s="2" t="n"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="n"/>
+      <c r="B250" s="2" t="n"/>
+      <c r="C250" s="2" t="n"/>
+      <c r="D250" s="2" t="n"/>
+      <c r="E250" s="3" t="n"/>
+      <c r="F250" s="2" t="n"/>
+      <c r="G250" s="2" t="n"/>
+      <c r="H250" s="2" t="n"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="n"/>
+      <c r="B251" s="2" t="n"/>
+      <c r="C251" s="2" t="n"/>
+      <c r="D251" s="2" t="n"/>
+      <c r="E251" s="3" t="n"/>
+      <c r="F251" s="2" t="n"/>
+      <c r="G251" s="2" t="n"/>
+      <c r="H251" s="2" t="n"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="n"/>
+      <c r="B252" s="2" t="n"/>
+      <c r="C252" s="2" t="n"/>
+      <c r="D252" s="2" t="n"/>
+      <c r="E252" s="3" t="n"/>
+      <c r="F252" s="2" t="n"/>
+      <c r="G252" s="2" t="n"/>
+      <c r="H252" s="2" t="n"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="n"/>
+      <c r="B253" s="2" t="n"/>
+      <c r="C253" s="2" t="n"/>
+      <c r="D253" s="2" t="n"/>
+      <c r="E253" s="3" t="n"/>
+      <c r="F253" s="2" t="n"/>
+      <c r="G253" s="2" t="n"/>
+      <c r="H253" s="2" t="n"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="n"/>
+      <c r="B254" s="2" t="n"/>
+      <c r="C254" s="2" t="n"/>
+      <c r="D254" s="2" t="n"/>
+      <c r="E254" s="3" t="n"/>
+      <c r="F254" s="2" t="n"/>
+      <c r="G254" s="2" t="n"/>
+      <c r="H254" s="2" t="n"/>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="n"/>
+      <c r="B255" s="2" t="n"/>
+      <c r="C255" s="2" t="n"/>
+      <c r="D255" s="2" t="n"/>
+      <c r="E255" s="3" t="n"/>
+      <c r="F255" s="2" t="n"/>
+      <c r="G255" s="2" t="n"/>
+      <c r="H255" s="2" t="n"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="n"/>
+      <c r="B256" s="2" t="n"/>
+      <c r="C256" s="2" t="n"/>
+      <c r="D256" s="2" t="n"/>
+      <c r="E256" s="3" t="n"/>
+      <c r="F256" s="2" t="n"/>
+      <c r="G256" s="2" t="n"/>
+      <c r="H256" s="2" t="n"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="n"/>
+      <c r="B257" s="2" t="n"/>
+      <c r="C257" s="2" t="n"/>
+      <c r="D257" s="2" t="n"/>
+      <c r="E257" s="3" t="n"/>
+      <c r="F257" s="2" t="n"/>
+      <c r="G257" s="2" t="n"/>
+      <c r="H257" s="2" t="n"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="n"/>
+      <c r="B258" s="2" t="n"/>
+      <c r="C258" s="2" t="n"/>
+      <c r="D258" s="2" t="n"/>
+      <c r="E258" s="3" t="n"/>
+      <c r="F258" s="2" t="n"/>
+      <c r="G258" s="2" t="n"/>
+      <c r="H258" s="2" t="n"/>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="n"/>
+      <c r="B259" s="2" t="n"/>
+      <c r="C259" s="2" t="n"/>
+      <c r="D259" s="2" t="n"/>
+      <c r="E259" s="3" t="n"/>
+      <c r="F259" s="2" t="n"/>
+      <c r="G259" s="2" t="n"/>
+      <c r="H259" s="2" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="n"/>
+      <c r="B260" s="2" t="n"/>
+      <c r="C260" s="2" t="n"/>
+      <c r="D260" s="2" t="n"/>
+      <c r="E260" s="3" t="n"/>
+      <c r="F260" s="2" t="n"/>
+      <c r="G260" s="2" t="n"/>
+      <c r="H260" s="2" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="n"/>
+      <c r="B261" s="2" t="n"/>
+      <c r="C261" s="2" t="n"/>
+      <c r="D261" s="2" t="n"/>
+      <c r="E261" s="3" t="n"/>
+      <c r="F261" s="2" t="n"/>
+      <c r="G261" s="2" t="n"/>
+      <c r="H261" s="2" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="n"/>
+      <c r="B262" s="2" t="n"/>
+      <c r="C262" s="2" t="n"/>
+      <c r="D262" s="2" t="n"/>
+      <c r="E262" s="3" t="n"/>
+      <c r="F262" s="2" t="n"/>
+      <c r="G262" s="2" t="n"/>
+      <c r="H262" s="2" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="n"/>
+      <c r="B263" s="2" t="n"/>
+      <c r="C263" s="2" t="n"/>
+      <c r="D263" s="2" t="n"/>
+      <c r="E263" s="3" t="n"/>
+      <c r="F263" s="2" t="n"/>
+      <c r="G263" s="2" t="n"/>
+      <c r="H263" s="2" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="n"/>
+      <c r="B264" s="2" t="n"/>
+      <c r="C264" s="2" t="n"/>
+      <c r="D264" s="2" t="n"/>
+      <c r="E264" s="3" t="n"/>
+      <c r="F264" s="2" t="n"/>
+      <c r="G264" s="2" t="n"/>
+      <c r="H264" s="2" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="n"/>
+      <c r="B265" s="2" t="n"/>
+      <c r="C265" s="2" t="n"/>
+      <c r="D265" s="2" t="n"/>
+      <c r="E265" s="3" t="n"/>
+      <c r="F265" s="2" t="n"/>
+      <c r="G265" s="2" t="n"/>
+      <c r="H265" s="2" t="n"/>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="n"/>
+      <c r="B266" s="2" t="n"/>
+      <c r="C266" s="2" t="n"/>
+      <c r="D266" s="2" t="n"/>
+      <c r="E266" s="3" t="n"/>
+      <c r="F266" s="2" t="n"/>
+      <c r="G266" s="2" t="n"/>
+      <c r="H266" s="2" t="n"/>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="n"/>
+      <c r="B267" s="2" t="n"/>
+      <c r="C267" s="2" t="n"/>
+      <c r="D267" s="2" t="n"/>
+      <c r="E267" s="3" t="n"/>
+      <c r="F267" s="2" t="n"/>
+      <c r="G267" s="2" t="n"/>
+      <c r="H267" s="2" t="n"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="n"/>
+      <c r="B268" s="2" t="n"/>
+      <c r="C268" s="2" t="n"/>
+      <c r="D268" s="2" t="n"/>
+      <c r="E268" s="3" t="n"/>
+      <c r="F268" s="2" t="n"/>
+      <c r="G268" s="2" t="n"/>
+      <c r="H268" s="2" t="n"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="n"/>
+      <c r="B269" s="2" t="n"/>
+      <c r="C269" s="2" t="n"/>
+      <c r="D269" s="2" t="n"/>
+      <c r="E269" s="3" t="n"/>
+      <c r="F269" s="2" t="n"/>
+      <c r="G269" s="2" t="n"/>
+      <c r="H269" s="2" t="n"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="n"/>
+      <c r="B270" s="2" t="n"/>
+      <c r="C270" s="2" t="n"/>
+      <c r="D270" s="2" t="n"/>
+      <c r="E270" s="3" t="n"/>
+      <c r="F270" s="2" t="n"/>
+      <c r="G270" s="2" t="n"/>
+      <c r="H270" s="2" t="n"/>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="n"/>
+      <c r="B271" s="2" t="n"/>
+      <c r="C271" s="2" t="n"/>
+      <c r="D271" s="2" t="n"/>
+      <c r="E271" s="3" t="n"/>
+      <c r="F271" s="2" t="n"/>
+      <c r="G271" s="2" t="n"/>
+      <c r="H271" s="2" t="n"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="n"/>
+      <c r="B272" s="2" t="n"/>
+      <c r="C272" s="2" t="n"/>
+      <c r="D272" s="2" t="n"/>
+      <c r="E272" s="3" t="n"/>
+      <c r="F272" s="2" t="n"/>
+      <c r="G272" s="2" t="n"/>
+      <c r="H272" s="2" t="n"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="n"/>
+      <c r="B273" s="2" t="n"/>
+      <c r="C273" s="2" t="n"/>
+      <c r="D273" s="2" t="n"/>
+      <c r="E273" s="3" t="n"/>
+      <c r="F273" s="2" t="n"/>
+      <c r="G273" s="2" t="n"/>
+      <c r="H273" s="2" t="n"/>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="n"/>
+      <c r="B274" s="2" t="n"/>
+      <c r="C274" s="2" t="n"/>
+      <c r="D274" s="2" t="n"/>
+      <c r="E274" s="3" t="n"/>
+      <c r="F274" s="2" t="n"/>
+      <c r="G274" s="2" t="n"/>
+      <c r="H274" s="2" t="n"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="n"/>
+      <c r="B275" s="2" t="n"/>
+      <c r="C275" s="2" t="n"/>
+      <c r="D275" s="2" t="n"/>
+      <c r="E275" s="3" t="n"/>
+      <c r="F275" s="2" t="n"/>
+      <c r="G275" s="2" t="n"/>
+      <c r="H275" s="2" t="n"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="n"/>
+      <c r="B276" s="2" t="n"/>
+      <c r="C276" s="2" t="n"/>
+      <c r="D276" s="2" t="n"/>
+      <c r="E276" s="3" t="n"/>
+      <c r="F276" s="2" t="n"/>
+      <c r="G276" s="2" t="n"/>
+      <c r="H276" s="2" t="n"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="n"/>
+      <c r="B277" s="2" t="n"/>
+      <c r="C277" s="2" t="n"/>
+      <c r="D277" s="2" t="n"/>
+      <c r="E277" s="3" t="n"/>
+      <c r="F277" s="2" t="n"/>
+      <c r="G277" s="2" t="n"/>
+      <c r="H277" s="2" t="n"/>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="n"/>
+      <c r="B278" s="2" t="n"/>
+      <c r="C278" s="2" t="n"/>
+      <c r="D278" s="2" t="n"/>
+      <c r="E278" s="3" t="n"/>
+      <c r="F278" s="2" t="n"/>
+      <c r="G278" s="2" t="n"/>
+      <c r="H278" s="2" t="n"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="n"/>
+      <c r="B279" s="2" t="n"/>
+      <c r="C279" s="2" t="n"/>
+      <c r="D279" s="2" t="n"/>
+      <c r="E279" s="3" t="n"/>
+      <c r="F279" s="2" t="n"/>
+      <c r="G279" s="2" t="n"/>
+      <c r="H279" s="2" t="n"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="n"/>
+      <c r="B280" s="2" t="n"/>
+      <c r="C280" s="2" t="n"/>
+      <c r="D280" s="2" t="n"/>
+      <c r="E280" s="3" t="n"/>
+      <c r="F280" s="2" t="n"/>
+      <c r="G280" s="2" t="n"/>
+      <c r="H280" s="2" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="n"/>
+      <c r="B281" s="2" t="n"/>
+      <c r="C281" s="2" t="n"/>
+      <c r="D281" s="2" t="n"/>
+      <c r="E281" s="3" t="n"/>
+      <c r="F281" s="2" t="n"/>
+      <c r="G281" s="2" t="n"/>
+      <c r="H281" s="2" t="n"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="n"/>
+      <c r="B282" s="2" t="n"/>
+      <c r="C282" s="2" t="n"/>
+      <c r="D282" s="2" t="n"/>
+      <c r="E282" s="3" t="n"/>
+      <c r="F282" s="2" t="n"/>
+      <c r="G282" s="2" t="n"/>
+      <c r="H282" s="2" t="n"/>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="n"/>
+      <c r="B283" s="2" t="n"/>
+      <c r="C283" s="2" t="n"/>
+      <c r="D283" s="2" t="n"/>
+      <c r="E283" s="3" t="n"/>
+      <c r="F283" s="2" t="n"/>
+      <c r="G283" s="2" t="n"/>
+      <c r="H283" s="2" t="n"/>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="n"/>
+      <c r="B284" s="2" t="n"/>
+      <c r="C284" s="2" t="n"/>
+      <c r="D284" s="2" t="n"/>
+      <c r="E284" s="3" t="n"/>
+      <c r="F284" s="2" t="n"/>
+      <c r="G284" s="2" t="n"/>
+      <c r="H284" s="2" t="n"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="n"/>
+      <c r="B285" s="2" t="n"/>
+      <c r="C285" s="2" t="n"/>
+      <c r="D285" s="2" t="n"/>
+      <c r="E285" s="3" t="n"/>
+      <c r="F285" s="2" t="n"/>
+      <c r="G285" s="2" t="n"/>
+      <c r="H285" s="2" t="n"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="n"/>
+      <c r="B286" s="2" t="n"/>
+      <c r="C286" s="2" t="n"/>
+      <c r="D286" s="2" t="n"/>
+      <c r="E286" s="3" t="n"/>
+      <c r="F286" s="2" t="n"/>
+      <c r="G286" s="2" t="n"/>
+      <c r="H286" s="2" t="n"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="n"/>
+      <c r="B287" s="2" t="n"/>
+      <c r="C287" s="2" t="n"/>
+      <c r="D287" s="2" t="n"/>
+      <c r="E287" s="3" t="n"/>
+      <c r="F287" s="2" t="n"/>
+      <c r="G287" s="2" t="n"/>
+      <c r="H287" s="2" t="n"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="n"/>
+      <c r="B288" s="2" t="n"/>
+      <c r="C288" s="2" t="n"/>
+      <c r="D288" s="2" t="n"/>
+      <c r="E288" s="3" t="n"/>
+      <c r="F288" s="2" t="n"/>
+      <c r="G288" s="2" t="n"/>
+      <c r="H288" s="2" t="n"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="n"/>
+      <c r="B289" s="2" t="n"/>
+      <c r="C289" s="2" t="n"/>
+      <c r="D289" s="2" t="n"/>
+      <c r="E289" s="3" t="n"/>
+      <c r="F289" s="2" t="n"/>
+      <c r="G289" s="2" t="n"/>
+      <c r="H289" s="2" t="n"/>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="n"/>
+      <c r="B290" s="2" t="n"/>
+      <c r="C290" s="2" t="n"/>
+      <c r="D290" s="2" t="n"/>
+      <c r="E290" s="3" t="n"/>
+      <c r="F290" s="2" t="n"/>
+      <c r="G290" s="2" t="n"/>
+      <c r="H290" s="2" t="n"/>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="n"/>
+      <c r="B291" s="2" t="n"/>
+      <c r="C291" s="2" t="n"/>
+      <c r="D291" s="2" t="n"/>
+      <c r="E291" s="3" t="n"/>
+      <c r="F291" s="2" t="n"/>
+      <c r="G291" s="2" t="n"/>
+      <c r="H291" s="2" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -6375,7 +9099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -6518,19 +9242,26 @@
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Dépenses : un total par mois (colonne « المصاريف الشهرية »), daté du dernier jour du mois (20 lignes).</t>
+          <t xml:space="preserve">  Dépenses : le détail de la feuille « المصاريف » — 84 salaires hebdomadaires du gardien et 6 recharges d'électricité (90 lignes).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Correction : « 31/06/2025 » (date inexistante) remplacé par 30/06/2025.</t>
+          <t xml:space="preserve">  Correction : semaine du 08/09 au 14/09 payée « 06/08/2025 » dans le fichier, remplacé par 06/09/2025 (à vérifier).</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Correction : « 31/06/2025 » (date inexistante) remplacé par 30/06/2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  Résultat attendu après les deux imports : solde en caisse 1 600,00 MAD au 10/10/2026, comme dans le fichier d'origine.</t>
         </is>

</xml_diff>